<commit_message>
Working dispatcher scout with Playwright
</commit_message>
<xml_diff>
--- a/output/dispatcher_jobs_tracker.xlsx
+++ b/output/dispatcher_jobs_tracker.xlsx
@@ -517,7 +517,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-09T12:34:43.270209+00:00</t>
+          <t>2026-05-09T13:23:54.068455+00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -588,7 +588,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-09T12:34:43.269304+00:00</t>
+          <t>2026-05-09T13:23:54.061995+00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-05-09T12:34:43.268437+00:00</t>
+          <t>2026-05-09T13:23:54.051531+00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-05-09T12:34:43.267210+00:00</t>
+          <t>2026-05-09T13:23:54.034221+00:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -797,11 +797,11 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-05-09T12:34:43.266228+00:00</t>
+          <t>2026-05-09T13:23:54.018467+00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -811,19 +811,19 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>flight dispatcher</t>
+          <t>aircraft dispatcher</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.jsfirm.com/allpositions/alltypes/allstates/allcountries/flight dispatcher/searchpopularjobs</t>
+          <t>https://www.jsfirm.com/allpositions/alltypes/allstates/allcountries/dispatcher/searchpopularjobs</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>flight dispatcher</t>
+          <t>aircraft dispatcher</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -854,6 +854,148 @@
       </c>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dear Hiring Team,
+I am applying for aircraft dispatcher with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
+My background includes leading 24/7 operations environments, managing large teams, improving service reliability, and responding to time-sensitive operational issues. I also bring aviation-specific training, FAR knowledge, private pilot experience, and a clear focus on dispatcher and flight operations work.
+What interests me about this role is the opportunity to support safe, reliable flight operations while building direct experience in airline, cargo, charter, or corporate aviation operations. I understand my transition point clearly: I am new to direct dispatch release work, but I bring mature operational judgment, communication discipline, and a strong safety mindset.
+I would welcome the opportunity to contribute to your operation and grow within your flight operations team.
+Sincerely,
+Ricky
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>15</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-05-09T13:23:54.018467+00:00</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>JSfirm Aircraft Dispatcher Search</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>aviation dispatcher</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>https://www.jsfirm.com/allpositions/alltypes/allstates/allcountries/aviation dispatcher/searchpopularjobs</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>aviation dispatcher</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>55</v>
+      </c>
+      <c r="L7" t="n">
+        <v>58</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dear Hiring Team,
+I am applying for aviation dispatcher with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
+My background includes leading 24/7 operations environments, managing large teams, improving service reliability, and responding to time-sensitive operational issues. I also bring aviation-specific training, FAR knowledge, private pilot experience, and a clear focus on dispatcher and flight operations work.
+What interests me about this role is the opportunity to support safe, reliable flight operations while building direct experience in airline, cargo, charter, or corporate aviation operations. I understand my transition point clearly: I am new to direct dispatch release work, but I bring mature operational judgment, communication discipline, and a strong safety mindset.
+I would welcome the opportunity to contribute to your operation and grow within your flight operations team.
+Sincerely,
+Ricky
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>16</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-05-09T13:23:54.018467+00:00</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>JSfirm Aircraft Dispatcher Search</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>flight dispatcher</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>https://www.jsfirm.com/allpositions/alltypes/allstates/allcountries/flight dispatcher/searchpopularjobs</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>flight dispatcher</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>55</v>
+      </c>
+      <c r="L8" t="n">
+        <v>58</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for flight dispatcher with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -866,68 +1008,68 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>15</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-05-09T12:34:43.265149+00:00</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="n">
+        <v>12</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-05-09T13:23:54.004753+00:00</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
         <is>
           <t>JSfirm Aircraft Dispatcher Search</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>aviation dispatcher</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>https://www.jsfirm.com/allpositions/alltypes/allstates/allcountries/aviation dispatcher/searchpopularjobs</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>aviation dispatcher</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Associate Flight Operations Generalist - Dispatcher</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>https://www.jsfirm.com/Dispatcher/Associate+Flight+Operations+Generalist+-+Dispatcher/Seattle-Washington/jobID_1937327</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Associate Flight Operations Generalist - Dispatcher</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Review manually</t>
         </is>
       </c>
-      <c r="K7" t="n">
+      <c r="K9" t="n">
         <v>55</v>
       </c>
-      <c r="L7" t="n">
+      <c r="L9" t="n">
         <v>58</v>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr">
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
-I am applying for aviation dispatcher with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
+I am applying for Associate Flight Operations Generalist - Dispatcher with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
 My background includes leading 24/7 operations environments, managing large teams, improving service reliability, and responding to time-sensitive operational issues. I also bring aviation-specific training, FAR knowledge, private pilot experience, and a clear focus on dispatcher and flight operations work.
 What interests me about this role is the opportunity to support safe, reliable flight operations while building direct experience in airline, cargo, charter, or corporate aviation operations. I understand my transition point clearly: I am new to direct dispatch release work, but I bring mature operational judgment, communication discipline, and a strong safety mindset.
 I would welcome the opportunity to contribute to your operation and grow within your flight operations team.
@@ -937,136 +1079,65 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>14</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-05-09T12:34:43.263954+00:00</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="n">
+        <v>13</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-05-09T13:23:54.004753+00:00</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
         <is>
           <t>JSfirm Aircraft Dispatcher Search</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>aircraft dispatcher</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>https://www.jsfirm.com/allpositions/alltypes/allstates/allcountries/dispatcher/searchpopularjobs</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>aircraft dispatcher</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Aircraft Dispatcher Program Coordinator</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://www.jsfirm.com/Dispatcher/Aircraft+Dispatcher+Program+Coordinator/Bloomington-Minnesota/jobID_1836221</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Aircraft Dispatcher Program Coordinator</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Review manually</t>
         </is>
       </c>
-      <c r="K8" t="n">
+      <c r="K10" t="n">
         <v>55</v>
       </c>
-      <c r="L8" t="n">
+      <c r="L10" t="n">
         <v>58</v>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dear Hiring Team,
-I am applying for aircraft dispatcher with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
-My background includes leading 24/7 operations environments, managing large teams, improving service reliability, and responding to time-sensitive operational issues. I also bring aviation-specific training, FAR knowledge, private pilot experience, and a clear focus on dispatcher and flight operations work.
-What interests me about this role is the opportunity to support safe, reliable flight operations while building direct experience in airline, cargo, charter, or corporate aviation operations. I understand my transition point clearly: I am new to direct dispatch release work, but I bring mature operational judgment, communication discipline, and a strong safety mindset.
-I would welcome the opportunity to contribute to your operation and grow within your flight operations team.
-Sincerely,
-Ricky
-</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>13</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-05-09T12:34:43.263305+00:00</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>JSfirm Aircraft Dispatcher Search</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Aircraft Dispatcher Program Coordinator</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>https://www.jsfirm.com/Dispatcher/Aircraft+Dispatcher+Program+Coordinator/Bloomington-Minnesota/jobID_1836221</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Aircraft Dispatcher Program Coordinator</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K9" t="n">
-        <v>55</v>
-      </c>
-      <c r="L9" t="n">
-        <v>58</v>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr">
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for Aircraft Dispatcher Program Coordinator with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -1079,84 +1150,13 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>12</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2026-05-09T12:34:43.262125+00:00</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>JSfirm Aircraft Dispatcher Search</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Associate Flight Operations Generalist - Dispatcher</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>https://www.jsfirm.com/Dispatcher/Associate+Flight+Operations+Generalist+-+Dispatcher/Seattle-Washington/jobID_1937327</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Associate Flight Operations Generalist - Dispatcher</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K10" t="n">
-        <v>55</v>
-      </c>
-      <c r="L10" t="n">
-        <v>58</v>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dear Hiring Team,
-I am applying for Associate Flight Operations Generalist - Dispatcher with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
-My background includes leading 24/7 operations environments, managing large teams, improving service reliability, and responding to time-sensitive operational issues. I also bring aviation-specific training, FAR knowledge, private pilot experience, and a clear focus on dispatcher and flight operations work.
-What interests me about this role is the opportunity to support safe, reliable flight operations while building direct experience in airline, cargo, charter, or corporate aviation operations. I understand my transition point clearly: I am new to direct dispatch release work, but I bring mature operational judgment, communication discipline, and a strong safety mindset.
-I would welcome the opportunity to contribute to your operation and grow within your flight operations team.
-Sincerely,
-Ricky
-</t>
-        </is>
-      </c>
-    </row>
     <row r="11">
       <c r="A11" t="n">
         <v>11</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-05-09T12:34:43.261272+00:00</t>
+          <t>2026-05-09T13:23:53.995137+00:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1223,11 +1223,11 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-05-09T12:34:43.260529+00:00</t>
+          <t>2026-05-09T13:23:53.971298+00:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1237,19 +1237,19 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Dispatcher - R0151301</t>
+          <t>Motor Vehicle Dispatcher</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.jsfirm.com/Dispatcher/Dispatcher+-+R0151301/McMurdo+Station-Ross+Island/jobID_1836049</t>
+          <t>https://www.jsfirm.com/Dispatcher/Motor+Vehicle+Dispatcher/Falls+Church-Virginia/jobID_1898982</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Dispatcher - R0151301</t>
+          <t>Motor Vehicle Dispatcher</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1280,6 +1280,148 @@
       </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dear Hiring Team,
+I am applying for Motor Vehicle Dispatcher with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
+My background includes leading 24/7 operations environments, managing large teams, improving service reliability, and responding to time-sensitive operational issues. I also bring aviation-specific training, FAR knowledge, private pilot experience, and a clear focus on dispatcher and flight operations work.
+What interests me about this role is the opportunity to support safe, reliable flight operations while building direct experience in airline, cargo, charter, or corporate aviation operations. I understand my transition point clearly: I am new to direct dispatch release work, but I bring mature operational judgment, communication discipline, and a strong safety mindset.
+I would welcome the opportunity to contribute to your operation and grow within your flight operations team.
+Sincerely,
+Ricky
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-05-09T13:23:53.971298+00:00</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>JSfirm Aircraft Dispatcher Search</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Part-Time Weekend Dispatcher, Motor Vehicle</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://www.jsfirm.com/Dispatcher/Part-Time+Weekend+Dispatcher,+Motor+Vehicle/Fort+Hood-Texas/jobID_1934031</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Part-Time Weekend Dispatcher, Motor Vehicle</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>55</v>
+      </c>
+      <c r="L13" t="n">
+        <v>58</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dear Hiring Team,
+I am applying for Part-Time Weekend Dispatcher, Motor Vehicle with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
+My background includes leading 24/7 operations environments, managing large teams, improving service reliability, and responding to time-sensitive operational issues. I also bring aviation-specific training, FAR knowledge, private pilot experience, and a clear focus on dispatcher and flight operations work.
+What interests me about this role is the opportunity to support safe, reliable flight operations while building direct experience in airline, cargo, charter, or corporate aviation operations. I understand my transition point clearly: I am new to direct dispatch release work, but I bring mature operational judgment, communication discipline, and a strong safety mindset.
+I would welcome the opportunity to contribute to your operation and grow within your flight operations team.
+Sincerely,
+Ricky
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-05-09T13:23:53.971298+00:00</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>JSfirm Aircraft Dispatcher Search</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Dispatcher - R0151301</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>https://www.jsfirm.com/Dispatcher/Dispatcher+-+R0151301/McMurdo+Station-Ross+Island/jobID_1836049</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Dispatcher - R0151301</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>55</v>
+      </c>
+      <c r="L14" t="n">
+        <v>58</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for Dispatcher - R0151301 with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -1292,155 +1434,13 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>2026-05-09T12:34:43.259467+00:00</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>JSfirm Aircraft Dispatcher Search</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Part-Time Weekend Dispatcher, Motor Vehicle</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>https://www.jsfirm.com/Dispatcher/Part-Time+Weekend+Dispatcher,+Motor+Vehicle/Fort+Hood-Texas/jobID_1934031</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Part-Time Weekend Dispatcher, Motor Vehicle</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K13" t="n">
-        <v>55</v>
-      </c>
-      <c r="L13" t="n">
-        <v>58</v>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dear Hiring Team,
-I am applying for Part-Time Weekend Dispatcher, Motor Vehicle with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
-My background includes leading 24/7 operations environments, managing large teams, improving service reliability, and responding to time-sensitive operational issues. I also bring aviation-specific training, FAR knowledge, private pilot experience, and a clear focus on dispatcher and flight operations work.
-What interests me about this role is the opportunity to support safe, reliable flight operations while building direct experience in airline, cargo, charter, or corporate aviation operations. I understand my transition point clearly: I am new to direct dispatch release work, but I bring mature operational judgment, communication discipline, and a strong safety mindset.
-I would welcome the opportunity to contribute to your operation and grow within your flight operations team.
-Sincerely,
-Ricky
-</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>8</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>2026-05-09T12:34:43.258647+00:00</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>JSfirm Aircraft Dispatcher Search</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Motor Vehicle Dispatcher</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>https://www.jsfirm.com/Dispatcher/Motor+Vehicle+Dispatcher/Falls+Church-Virginia/jobID_1898982</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Motor Vehicle Dispatcher</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K14" t="n">
-        <v>55</v>
-      </c>
-      <c r="L14" t="n">
-        <v>58</v>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dear Hiring Team,
-I am applying for Motor Vehicle Dispatcher with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
-My background includes leading 24/7 operations environments, managing large teams, improving service reliability, and responding to time-sensitive operational issues. I also bring aviation-specific training, FAR knowledge, private pilot experience, and a clear focus on dispatcher and flight operations work.
-What interests me about this role is the opportunity to support safe, reliable flight operations while building direct experience in airline, cargo, charter, or corporate aviation operations. I understand my transition point clearly: I am new to direct dispatch release work, but I bring mature operational judgment, communication discipline, and a strong safety mindset.
-I would welcome the opportunity to contribute to your operation and grow within your flight operations team.
-Sincerely,
-Ricky
-</t>
-        </is>
-      </c>
-    </row>
     <row r="15">
       <c r="A15" t="n">
         <v>7</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-05-09T12:34:43.257424+00:00</t>
+          <t>2026-05-09T13:23:53.964785+00:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-05-09T12:34:43.256505+00:00</t>
+          <t>2026-05-09T13:23:53.955228+00:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-05-09T12:34:43.255765+00:00</t>
+          <t>2026-05-09T13:23:53.944260+00:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-05-09T12:34:43.254634+00:00</t>
+          <t>2026-05-09T13:23:53.938519+00:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1724,7 +1724,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-05-09T12:34:43.253781+00:00</t>
+          <t>2026-05-09T13:23:53.932505+00:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1795,7 +1795,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-05-09T12:34:43.252933+00:00</t>
+          <t>2026-05-09T13:23:53.928480+00:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-05-09T12:34:43.251789+00:00</t>
+          <t>2026-05-09T13:23:53.909888+00:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2005,7 +2005,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-05-09T12:52:23.126938+00:00</t>
+          <t>2026-05-09T13:23:54.368435+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix scout syntax and run locally
</commit_message>
<xml_diff>
--- a/output/dispatcher_jobs_tracker.xlsx
+++ b/output/dispatcher_jobs_tracker.xlsx
@@ -1942,7 +1942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1990,22 +1990,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>New jobs</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
           <t>Last run UTC</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-05-09T13:23:54.368435+00:00</t>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-05-09T13:45:58.469781+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dispatcher job scout results
</commit_message>
<xml_diff>
--- a/output/dispatcher_jobs_tracker.xlsx
+++ b/output/dispatcher_jobs_tracker.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="Job Tracker" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -426,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:P23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,63 +512,183 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-09T13:23:54.068455+00:00</t>
+          <t>2026-05-09T14:31:43.351023+00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>JSfirm Aircraft Dispatcher Search</t>
+          <t>Mountain Air Cargo Openings</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Aircraft Dispatcher Jobs</t>
+          <t>Flight Follower/Dispatcher</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
+          <t>job-opening.php?req=2795320&amp;req_loc=274806&amp;&amp;cust_sort1=170262&amp;#job</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Flight Follower/Dispatcher</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>65</v>
+      </c>
+      <c r="L2" t="n">
+        <v>68</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-05-09T14:31:43.351023+00:00</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Piedmont Airlines Operations Careers</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Flight Operations Jobs</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>https://piedmont-airlines.com/other-careers/operations/</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Flight Operations Jobs</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>45</v>
+      </c>
+      <c r="L3" t="n">
+        <v>48</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-05-09T13:23:54.068455+00:00</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>JSfirm Aircraft Dispatcher Search</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Aircraft Dispatcher Jobs</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>https://www.jsfirm.com/aircraft+dispatcher+jobs</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Aircraft Dispatcher Jobs</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
         <v>55</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L4" t="n">
         <v>58</v>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr">
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for Aircraft Dispatcher Jobs with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -582,65 +701,65 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="n">
+    <row r="5">
+      <c r="A5" t="n">
         <v>19</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>2026-05-09T13:23:54.061995+00:00</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>JSfirm Aircraft Dispatcher Search</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Aircraft Dispatcher Jobs Overseas</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
         <is>
           <t>https://www.jsfirm.com/all positions/alltypes/allstates/International/dispatcher/searchpopularjobs</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Aircraft Dispatcher Jobs Overseas</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K3" t="n">
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
         <v>55</v>
       </c>
-      <c r="L3" t="n">
+      <c r="L5" t="n">
         <v>58</v>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr">
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for Aircraft Dispatcher Jobs Overseas with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -653,65 +772,65 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="n">
+    <row r="6">
+      <c r="A6" t="n">
         <v>18</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>2026-05-09T13:23:54.051531+00:00</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>JSfirm Aircraft Dispatcher Search</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>aircraft flight dispatcher</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
         <is>
           <t>https://www.jsfirm.com/allpositions/alltypes/allstates/allcountries/aircraft flight dispatcher/searchpopularjobs</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>aircraft flight dispatcher</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
         <v>55</v>
       </c>
-      <c r="L4" t="n">
+      <c r="L6" t="n">
         <v>58</v>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr">
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for aircraft flight dispatcher with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -724,65 +843,65 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="n">
+    <row r="7">
+      <c r="A7" t="n">
         <v>17</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>2026-05-09T13:23:54.034221+00:00</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>JSfirm Aircraft Dispatcher Search</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>flight follower</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
         <is>
           <t>https://www.jsfirm.com/allpositions/alltypes/allstates/allcountries/flight follower/searchpopularjobs</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>flight follower</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
         <v>63</v>
       </c>
-      <c r="L5" t="n">
+      <c r="L7" t="n">
         <v>66</v>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr">
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for flight follower with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -795,65 +914,65 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="n">
+    <row r="8">
+      <c r="A8" t="n">
         <v>14</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>2026-05-09T13:23:54.018467+00:00</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>JSfirm Aircraft Dispatcher Search</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>aircraft dispatcher</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
         <is>
           <t>https://www.jsfirm.com/allpositions/alltypes/allstates/allcountries/dispatcher/searchpopularjobs</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>aircraft dispatcher</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
         <v>55</v>
       </c>
-      <c r="L6" t="n">
+      <c r="L8" t="n">
         <v>58</v>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr">
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for aircraft dispatcher with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -866,65 +985,65 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="n">
+    <row r="9">
+      <c r="A9" t="n">
         <v>15</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>2026-05-09T13:23:54.018467+00:00</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>JSfirm Aircraft Dispatcher Search</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>aviation dispatcher</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
         <is>
           <t>https://www.jsfirm.com/allpositions/alltypes/allstates/allcountries/aviation dispatcher/searchpopularjobs</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>aviation dispatcher</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K7" t="n">
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
         <v>55</v>
       </c>
-      <c r="L7" t="n">
+      <c r="L9" t="n">
         <v>58</v>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr">
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for aviation dispatcher with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -937,65 +1056,65 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="n">
+    <row r="10">
+      <c r="A10" t="n">
         <v>16</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>2026-05-09T13:23:54.018467+00:00</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>JSfirm Aircraft Dispatcher Search</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>flight dispatcher</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
         <is>
           <t>https://www.jsfirm.com/allpositions/alltypes/allstates/allcountries/flight dispatcher/searchpopularjobs</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>flight dispatcher</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K8" t="n">
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
         <v>55</v>
       </c>
-      <c r="L8" t="n">
+      <c r="L10" t="n">
         <v>58</v>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr">
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for flight dispatcher with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -1008,65 +1127,65 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="n">
+    <row r="11">
+      <c r="A11" t="n">
         <v>12</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>2026-05-09T13:23:54.004753+00:00</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>JSfirm Aircraft Dispatcher Search</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Associate Flight Operations Generalist - Dispatcher</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
         <is>
           <t>https://www.jsfirm.com/Dispatcher/Associate+Flight+Operations+Generalist+-+Dispatcher/Seattle-Washington/jobID_1937327</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>Associate Flight Operations Generalist - Dispatcher</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K9" t="n">
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
         <v>55</v>
       </c>
-      <c r="L9" t="n">
+      <c r="L11" t="n">
         <v>58</v>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr">
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for Associate Flight Operations Generalist - Dispatcher with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -1079,65 +1198,65 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="n">
+    <row r="12">
+      <c r="A12" t="n">
         <v>13</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>2026-05-09T13:23:54.004753+00:00</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>JSfirm Aircraft Dispatcher Search</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Aircraft Dispatcher Program Coordinator</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
         <is>
           <t>https://www.jsfirm.com/Dispatcher/Aircraft+Dispatcher+Program+Coordinator/Bloomington-Minnesota/jobID_1836221</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>Aircraft Dispatcher Program Coordinator</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K10" t="n">
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
         <v>55</v>
       </c>
-      <c r="L10" t="n">
+      <c r="L12" t="n">
         <v>58</v>
       </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr">
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for Aircraft Dispatcher Program Coordinator with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -1150,65 +1269,65 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="n">
+    <row r="13">
+      <c r="A13" t="n">
         <v>11</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>2026-05-09T13:23:53.995137+00:00</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>JSfirm Aircraft Dispatcher Search</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Dispatcher Lead - R0151304</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr">
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
         <is>
           <t>https://www.jsfirm.com/Dispatcher/Dispatcher+Lead+-+R0151304/McMurdo+Station-Ross+Island/jobID_1836046</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>Dispatcher Lead - R0151304</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K11" t="n">
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
         <v>55</v>
       </c>
-      <c r="L11" t="n">
+      <c r="L13" t="n">
         <v>58</v>
       </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr">
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for Dispatcher Lead - R0151304 with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -1221,65 +1340,65 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="n">
+    <row r="14">
+      <c r="A14" t="n">
         <v>8</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>2026-05-09T13:23:53.971298+00:00</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>JSfirm Aircraft Dispatcher Search</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Motor Vehicle Dispatcher</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr">
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
         <is>
           <t>https://www.jsfirm.com/Dispatcher/Motor+Vehicle+Dispatcher/Falls+Church-Virginia/jobID_1898982</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>Motor Vehicle Dispatcher</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K12" t="n">
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
         <v>55</v>
       </c>
-      <c r="L12" t="n">
+      <c r="L14" t="n">
         <v>58</v>
       </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr">
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for Motor Vehicle Dispatcher with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -1292,65 +1411,65 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="n">
+    <row r="15">
+      <c r="A15" t="n">
         <v>9</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>2026-05-09T13:23:53.971298+00:00</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>JSfirm Aircraft Dispatcher Search</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>Part-Time Weekend Dispatcher, Motor Vehicle</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr">
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
         <is>
           <t>https://www.jsfirm.com/Dispatcher/Part-Time+Weekend+Dispatcher,+Motor+Vehicle/Fort+Hood-Texas/jobID_1934031</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>Part-Time Weekend Dispatcher, Motor Vehicle</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K13" t="n">
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
         <v>55</v>
       </c>
-      <c r="L13" t="n">
+      <c r="L15" t="n">
         <v>58</v>
       </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr">
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for Part-Time Weekend Dispatcher, Motor Vehicle with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -1363,65 +1482,65 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="n">
+    <row r="16">
+      <c r="A16" t="n">
         <v>10</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>2026-05-09T13:23:53.971298+00:00</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>JSfirm Aircraft Dispatcher Search</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Dispatcher - R0151301</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr">
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
         <is>
           <t>https://www.jsfirm.com/Dispatcher/Dispatcher+-+R0151301/McMurdo+Station-Ross+Island/jobID_1836049</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>Dispatcher - R0151301</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K14" t="n">
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
         <v>55</v>
       </c>
-      <c r="L14" t="n">
+      <c r="L16" t="n">
         <v>58</v>
       </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr">
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for Dispatcher - R0151301 with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -1434,65 +1553,65 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="n">
+    <row r="17">
+      <c r="A17" t="n">
         <v>7</v>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>2026-05-09T13:23:53.964785+00:00</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>JSfirm Aircraft Dispatcher Search</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Motor Vehicle Dispatcher (Must have Secret Clearance)</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr">
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
         <is>
           <t>https://www.jsfirm.com/Other/Motor+Vehicle+Dispatcher+(Must+have+Secret+Clearance)/Arlington-Virginia/jobID_1756119</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>Motor Vehicle Dispatcher (Must have Secret Clearance)</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K15" t="n">
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
         <v>55</v>
       </c>
-      <c r="L15" t="n">
+      <c r="L17" t="n">
         <v>58</v>
       </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr">
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for Motor Vehicle Dispatcher (Must have Secret Clearance) with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -1505,65 +1624,65 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="n">
+    <row r="18">
+      <c r="A18" t="n">
         <v>6</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>2026-05-09T13:23:53.955228+00:00</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>JSfirm Aircraft Dispatcher Search</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>Shuttle Bus Dispatcher - Part Time</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr">
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
         <is>
           <t>https://www.jsfirm.com/Other/Shuttle+Bus+Dispatcher+-+Part+Time/Indianapolis-Indiana/jobID_1940552</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>Shuttle Bus Dispatcher - Part Time</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K16" t="n">
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
         <v>55</v>
       </c>
-      <c r="L16" t="n">
+      <c r="L18" t="n">
         <v>58</v>
       </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr">
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for Shuttle Bus Dispatcher - Part Time with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -1576,65 +1695,65 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="n">
+    <row r="19">
+      <c r="A19" t="n">
         <v>5</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>2026-05-09T13:23:53.944260+00:00</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>JSfirm Aircraft Dispatcher Search</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>Aircraft Dispatcher Apprenticeship</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr">
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
         <is>
           <t>https://www.jsfirm.com/Dispatcher/Aircraft+Dispatcher+Apprenticeship/Indianapolis-Indiana/jobID_1920604</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>Aircraft Dispatcher Apprenticeship</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K17" t="n">
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
         <v>55</v>
       </c>
-      <c r="L17" t="n">
+      <c r="L19" t="n">
         <v>58</v>
       </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr">
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for Aircraft Dispatcher Apprenticeship with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -1647,65 +1766,65 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="n">
+    <row r="20">
+      <c r="A20" t="n">
         <v>4</v>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>2026-05-09T13:23:53.938519+00:00</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>JSfirm Aircraft Dispatcher Search</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Flight Follower/Dispatcher</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
         <is>
           <t>https://www.jsfirm.com/Dispatcher/Flight+Follower/Dispatcher/Denver-North+Carolina/jobID_1283517</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>Flight Follower/Dispatcher</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K18" t="n">
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
         <v>63</v>
       </c>
-      <c r="L18" t="n">
+      <c r="L20" t="n">
         <v>66</v>
       </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr">
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for Flight Follower/Dispatcher with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -1718,65 +1837,65 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="n">
+    <row r="21">
+      <c r="A21" t="n">
         <v>3</v>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>2026-05-09T13:23:53.932505+00:00</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>JSfirm Aircraft Dispatcher Search</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>Dispatcher</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
         <is>
           <t>https://www.jsfirm.com/Dispatcher/Dispatcher/Denver-Colorado/jobID_1934127</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>Dispatcher</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K19" t="n">
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
         <v>55</v>
       </c>
-      <c r="L19" t="n">
+      <c r="L21" t="n">
         <v>58</v>
       </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr">
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for Dispatcher with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -1789,65 +1908,65 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="n">
+    <row r="22">
+      <c r="A22" t="n">
         <v>2</v>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>2026-05-09T13:23:53.928480+00:00</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>JSfirm Aircraft Dispatcher Search</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Aircraft Dispatcher</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr">
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
         <is>
           <t>https://www.jsfirm.com/Dispatcher/Aircraft+Dispatcher/Charlotte-North+Carolina/jobID_1869294</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>Aircraft Dispatcher</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K20" t="n">
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
         <v>55</v>
       </c>
-      <c r="L20" t="n">
+      <c r="L22" t="n">
         <v>58</v>
       </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr">
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for Aircraft Dispatcher with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -1860,65 +1979,65 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="n">
+    <row r="23">
+      <c r="A23" t="n">
         <v>1</v>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>2026-05-09T13:23:53.909888+00:00</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>JSfirm Aircraft Dispatcher Search</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>AOG Maintenance Controller (Dispatcher) - Night Shift</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
         <is>
           <t>https://www.jsfirm.com/Administration/AOG+Maintenance+Controller+(Dispatcher)+-+Night+Shift/Kinston-North+Carolina/jobID_1690983</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>AOG Maintenance Controller (Dispatcher) - Night Shift</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>Review manually</t>
-        </is>
-      </c>
-      <c r="K21" t="n">
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Review manually</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
         <v>55</v>
       </c>
-      <c r="L21" t="n">
+      <c r="L23" t="n">
         <v>58</v>
       </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr">
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
         <is>
           <t xml:space="preserve">Dear Hiring Team,
 I am applying for AOG Maintenance Controller (Dispatcher) - Night Shift with . I hold an FAA Aircraft Dispatcher Certificate and bring a strong operations background built around real-time decision making, safety, compliance, and coordination across teams.
@@ -1934,72 +2053,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Total jobs</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Very High priority</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>High priority</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Last run UTC</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-05-09T13:53:23.265296+00:00</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>